<commit_message>
Refactor quality control Excel import/export functionality
- Updated the Excel export process to utilize a shared wizard for exporting quality tests, ensuring consistency and reducing code duplication.
- Enhanced the import functionality to accommodate new header structures and improved data handling for qualitative and quantitative questions.
- Modified the test cases to validate the new import/export logic, ensuring that all relevant fields are correctly processed and mapped.
- Adjusted the UI elements to reflect changes in the export action, providing a more intuitive user experience.
- Improved error handling and validation during the import process to ensure data integrity and user feedback.
</commit_message>
<xml_diff>
--- a/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
+++ b/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
@@ -1,30 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl"/>
-  <workbookPr date1904="0"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13200"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Product Test Template" sheetId="1" r:id="rId1"/>
+    <sheet name="Quality Tests" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -43,46 +47,404 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>product_template_default_code</t>
+          <t>trigger_product_template_line_ids/product_template/default_code</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>product_template_name</t>
+          <t>trigger_product_template_line_ids/product_template/name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>test_code</t>
+          <t>code</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>test_name</t>
+          <t>name</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>test_type</t>
+          <t>type</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>test_category_xmlid</t>
+          <t>category/id</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -92,62 +454,62 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>trigger_name</t>
+          <t>trigger_product_template_line_ids/trigger/name</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>trigger_timing</t>
+          <t>trigger_product_template_line_ids/timing</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>question_sequence</t>
+          <t>test_lines/sequence</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>question_code</t>
+          <t>test_lines/code</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>question_name</t>
+          <t>test_lines/name</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>question_type</t>
+          <t>test_lines/type</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>question_notes</t>
+          <t>test_lines/notes</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>uom_xmlid</t>
+          <t>test_lines/uom_id/id</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>min_value</t>
+          <t>test_lines/min_value</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>max_value</t>
+          <t>test_lines/max_value</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>qualitative_value_name</t>
+          <t>test_lines/ql_values/name</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>qualitative_value_ok</t>
+          <t>test_lines/ql_values/ok</t>
         </is>
       </c>
     </row>
@@ -195,7 +557,7 @@
           <t>after</t>
         </is>
       </c>
-      <c r="J2">
+      <c r="J2" t="n">
         <v>10</v>
       </c>
       <c r="K2" t="inlineStr">
@@ -223,14 +585,12 @@
           <t>uom.product_uom_celsius</t>
         </is>
       </c>
-      <c r="P2">
+      <c r="P2" t="n">
         <v>120</v>
       </c>
-      <c r="Q2">
+      <c r="Q2" t="n">
         <v>130</v>
       </c>
-      <c r="R2"/>
-      <c r="S2"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -276,7 +636,7 @@
           <t>after</t>
         </is>
       </c>
-      <c r="J3">
+      <c r="J3" t="n">
         <v>20</v>
       </c>
       <c r="K3" t="inlineStr">
@@ -299,9 +659,6 @@
           <t>Visual inspection</t>
         </is>
       </c>
-      <c r="O3"/>
-      <c r="P3"/>
-      <c r="Q3"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>Clear</t>
@@ -355,7 +712,7 @@
           <t>after</t>
         </is>
       </c>
-      <c r="J4">
+      <c r="J4" t="n">
         <v>20</v>
       </c>
       <c r="K4" t="inlineStr">
@@ -378,9 +735,6 @@
           <t>Visual inspection</t>
         </is>
       </c>
-      <c r="O4"/>
-      <c r="P4"/>
-      <c r="Q4"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>Amber</t>
@@ -391,5 +745,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: I simplified the wizard and cleaned up the template so that you can import question sets without having to deal with side data such as triggers or UoM.
</commit_message>
<xml_diff>
--- a/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
+++ b/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
@@ -413,7 +413,7 @@
     <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
     <ns0:pageSetUpPr/>
   </ns0:sheetPr>
-  <ns0:dimension ref="A1:U4"/>
+  <ns0:dimension ref="A1:U1"/>
   <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <ns0:sheetData>
     <ns0:row r="1">
@@ -521,257 +521,6 @@
         <ns0:is>
           <ns0:t>test_lines/ql_values/ok</ns0:t>
         </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="2">
-      <ns0:c r="A2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>FERT-001</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sterilized Filter</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>STERIL_TEST</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sterility Check</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>related</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>quality_control_oca.qc_test_category_process</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Process</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H2" t="b">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="I2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Manufacturing Order</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>after</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K2">
-        <ns0:v>10</ns0:v>
-      </ns0:c>
-      <ns0:c r="L2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>STER_TEMP</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sterilization Temperature</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>quantitative</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Target range 120-130 C</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="P2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>uom.product_uom_celsius</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="Q2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Degrees Celsius</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="R2">
-        <ns0:v>120</ns0:v>
-      </ns0:c>
-      <ns0:c r="S2">
-        <ns0:v>130</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3">
-      <ns0:c r="A3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>FERT-001</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sterilized Filter</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>STERIL_TEST</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sterility Check</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>related</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>quality_control_oca.qc_test_category_process</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Process</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H3" t="b">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Manufacturing Order</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>after</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K3">
-        <ns0:v>20</ns0:v>
-      </ns0:c>
-      <ns0:c r="L3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>STER_COLOR</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Filter Color</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>qualitative</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Visual inspection</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="T3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Clear</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="U3" t="b">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4">
-      <ns0:c r="A4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>FERT-001</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sterilized Filter</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>STERIL_TEST</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sterility Check</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>related</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>quality_control_oca.qc_test_category_process</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Process</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H4" t="b">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Manufacturing Order</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>after</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K4">
-        <ns0:v>20</ns0:v>
-      </ns0:c>
-      <ns0:c r="L4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>STER_COLOR</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Filter Color</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>qualitative</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Visual inspection</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="T4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Amber</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="U4" t="b">
-        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
   </ns0:sheetData>

</xml_diff>

<commit_message>
feat: update sample file.
</commit_message>
<xml_diff>
--- a/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
+++ b/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
@@ -408,122 +408,159 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:sheetPr>
-    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
-    <ns0:pageSetUpPr/>
-  </ns0:sheetPr>
-  <ns0:dimension ref="A1:U1"/>
-  <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <ns0:sheetData>
-    <ns0:row r="1">
-      <ns0:c r="A1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>trigger_product_template_line_ids/product_template/default_code</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>trigger_product_template_line_ids/product_template/name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>code</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>type</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>category/id</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>category/name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>fill_correct_values</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="I1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>trigger_product_template_line_ids/trigger/name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>trigger_product_template_line_ids/timing</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/sequence</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="L1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/code</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/type</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/notes</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="P1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/uom_id/id</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="Q1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/uom_id/name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="R1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/min_value</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="S1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/max_value</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="T1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/ql_values/name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="U1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>test_lines/ql_values/ok</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>test_lines/sequence</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>test_lines/name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>test_lines/type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>test_lines/ql_values/name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>test_lines/ql_values/ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Elektronik Kontrol Testi</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>LCD ekran kontrolü</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Elektronik Kontrol Testi</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LCD ekran kontrolü</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Elektronik Kontrol Testi</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Görev PWM HZ Kontrolü</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Uyumlu</t>
+        </is>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Elektronik Kontrol Testi</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Görev PWM HZ Kontrolü</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Uyumsuz</t>
+        </is>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: update QC product questions template Excel file
</commit_message>
<xml_diff>
--- a/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
+++ b/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
   <si>
     <t>name</t>
   </si>
@@ -43,16 +43,10 @@
     <t>test_lines/uom</t>
   </si>
   <si>
-    <t>PCB Name</t>
-  </si>
-  <si>
     <t>test</t>
   </si>
   <si>
-    <t>qualitative</t>
-  </si>
-  <si>
-    <t>Check the PCB surface for scratches</t>
+    <t>Test Question</t>
   </si>
   <si>
     <t>OK</t>
@@ -61,13 +55,13 @@
     <t>true</t>
   </si>
   <si>
-    <t>test1</t>
-  </si>
-  <si>
-    <t>NOK</t>
+    <t>Not OK</t>
   </si>
   <si>
     <t>false</t>
+  </si>
+  <si>
+    <t>Test1 Question</t>
   </si>
 </sst>
 </file>
@@ -414,15 +408,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="2" width="30.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="29.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="26.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="42.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="22.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="2" width="24.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="2" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="2" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="2" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="2" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="2" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="2" width="13.005" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="2" width="13.005" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="2" width="13.005" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="2" width="13.005" customWidth="1" bestFit="1"/>
@@ -464,17 +458,13 @@
       <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -485,23 +475,57 @@
         <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+      <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: improve active_ids handling in export wizard and update product questions template
</commit_message>
<xml_diff>
--- a/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
+++ b/quality_control_oca/static/xlsx/qc_product_questions_template.xlsx
@@ -1,86 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Quality Tests"/>
+    <sheet name="Quality Tests" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>test_lines/name</t>
-  </si>
-  <si>
-    <t>test_lines/type</t>
-  </si>
-  <si>
-    <t>test_lines/notes</t>
-  </si>
-  <si>
-    <t>test_lines/ql_values/name</t>
-  </si>
-  <si>
-    <t>test_lines/ql_values/ok</t>
-  </si>
-  <si>
-    <t>test_lines/min_value</t>
-  </si>
-  <si>
-    <t>test_lines/max_value</t>
-  </si>
-  <si>
-    <t>test_lines/uom</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>Test Question</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>Not OK</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>Test1 Question</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -99,24 +46,86 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -404,128 +413,171 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="2" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="2" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="2" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="2" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="2" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="2" width="13.005" customWidth="1" bestFit="1"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="2" min="5" max="5"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="2" min="7" max="7"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="2" min="8" max="8"/>
+    <col width="13.005" bestFit="1" customWidth="1" style="2" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>test_lines/name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>test_lines/type</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>test_lines/notes</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>test_lines/ql_values/name</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>test_lines/ql_values/ok</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>test_lines/min_value</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>test_lines/max_value</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>test_lines/uom</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Test Question</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Test Question</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Not OK</t>
+        </is>
+      </c>
+      <c r="F3" t="b">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Test1 Question</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F4" t="b">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Test1 Question</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Not OK</t>
+        </is>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>